<commit_message>
Update Available Unused Functions.xlsx
Updated
</commit_message>
<xml_diff>
--- a/MapFiles/Available Unused Functions.xlsx
+++ b/MapFiles/Available Unused Functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Den\OneDrive\Personal\Thrustmaster\TARGET\Clicker\Development\ED_Enhanced_T16000\MapFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C34686E0-D774-4E45-8139-67DC81A480DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85651F5-6E4B-409D-B150-EFC4B9C47582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11265" yWindow="720" windowWidth="24870" windowHeight="20235" xr2:uid="{E4944AEC-5D5F-4A78-AAD3-49930FCA7BF6}"/>
+    <workbookView xWindow="5370" yWindow="345" windowWidth="29115" windowHeight="20235" xr2:uid="{E4944AEC-5D5F-4A78-AAD3-49930FCA7BF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>T16000 Enhanced TARGET Script</t>
   </si>
@@ -44,36 +44,15 @@
     <t>Underused Functions</t>
   </si>
   <si>
-    <t>fnFlashLED</t>
-  </si>
-  <si>
-    <t>fnSetLEDs</t>
-  </si>
-  <si>
-    <t>fnFlashStart</t>
-  </si>
-  <si>
     <t>Action</t>
   </si>
   <si>
-    <t>Remove</t>
-  </si>
-  <si>
     <t>Keep</t>
   </si>
   <si>
     <t>fnDeploySRV</t>
   </si>
   <si>
-    <t>fnIdleLock</t>
-  </si>
-  <si>
-    <t>fnDebug</t>
-  </si>
-  <si>
-    <t>fnGetDate</t>
-  </si>
-  <si>
     <t>m_DeploySRV</t>
   </si>
   <si>
@@ -83,19 +62,10 @@
     <t>m_Launch</t>
   </si>
   <si>
-    <t>stfnDumpFlags</t>
-  </si>
-  <si>
-    <t>stfnDumpFlags2</t>
-  </si>
-  <si>
     <t>tgTxt2Speech</t>
   </si>
   <si>
     <t>m_BoardShip</t>
-  </si>
-  <si>
-    <t>fnLEDBrightness</t>
   </si>
 </sst>
 </file>
@@ -111,18 +81,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -146,11 +110,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A98F157-F02E-49C6-B982-A51895D99908}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
@@ -501,128 +463,56 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" thickTop="1"/>
     <row r="5" spans="1:2">
-      <c r="A5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="2" t="s">
+      <c r="B10" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="3" t="s">
+      <c r="A11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B22" t="s">
-        <v>7</v>
+      <c r="B11" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>